<commit_message>
add homework1 to week-02
</commit_message>
<xml_diff>
--- a/week-01/Ex2B_data_roundup.xlsx
+++ b/week-01/Ex2B_data_roundup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kendratyler\Documents\dataanalytics\week-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B763AE7D-F8EE-40E2-BF9C-927B4E48D885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B85FB72-31AF-43E5-9647-20C00288E818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{420B7977-4B87-4A86-8DC3-08F8B96D72E4}"/>
+    <workbookView xWindow="3720" yWindow="460" windowWidth="11990" windowHeight="11220" xr2:uid="{420B7977-4B87-4A86-8DC3-08F8B96D72E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
   <si>
     <t xml:space="preserve">Name of data soucre </t>
   </si>
@@ -57,6 +57,39 @@
   </si>
   <si>
     <t xml:space="preserve">Additional notes </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Instagram </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Photos &amp; Vidoes </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Creation of account </t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Go to settings &amp; Privacy &gt; Settings&gt; Account Center &gt; Your Information and premission &gt; Download your information. Select 'posts' or "photos and videos" and Click "Submit Request"</t>
+  </si>
+  <si>
+    <t>Zip File</t>
+  </si>
+  <si>
+    <t>GitBash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data Analytics classwork documents </t>
+  </si>
+  <si>
+    <t>1.Navigate to the main page of your repository on GitHub.         2. Clickthe green Code buttton loacted above the file list.           3. Select Download ZIP from the dropdwon menu.                                 4. Once downloaded, locate the ZIP file on your computer and extract its contents to access your documents.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Procreate </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Digital Art </t>
   </si>
 </sst>
 </file>
@@ -92,8 +125,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -428,14 +464,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35003B15-8E25-4BAC-A2BA-C8C09A1664BA}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.81640625" customWidth="1"/>
-    <col min="2" max="2" width="11.54296875" customWidth="1"/>
-    <col min="3" max="3" width="15.6328125" customWidth="1"/>
+    <col min="2" max="2" width="30.54296875" customWidth="1"/>
+    <col min="3" max="3" width="20.54296875" customWidth="1"/>
     <col min="4" max="4" width="14.453125" customWidth="1"/>
-    <col min="5" max="5" width="16.08984375" customWidth="1"/>
+    <col min="5" max="5" width="25.7265625" customWidth="1"/>
     <col min="6" max="6" width="14.6328125" customWidth="1"/>
     <col min="7" max="7" width="22.1796875" customWidth="1"/>
   </cols>
@@ -463,6 +499,63 @@
         <v>6</v>
       </c>
     </row>
+    <row r="2" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="145" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>